<commit_message>
auto reload is added so time for my ass to fix all the ugly asf css
</commit_message>
<xml_diff>
--- a/CLIENT_FEEDBACK.xlsx
+++ b/CLIENT_FEEDBACK.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -609,6 +609,61 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-17 23:30:52</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>qwdqwd12d12d</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>qwdqwdqwd12d</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>user@example.com</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>87654321</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed all css, left changing everything to bootstrap
</commit_message>
<xml_diff>
--- a/CLIENT_FEEDBACK.xlsx
+++ b/CLIENT_FEEDBACK.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,116 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-18 06:39:16</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>qwdqwdqwd</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>qwdqwd1212das</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-18 06:40:44</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>improvement</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>qwdqwdqw1212</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>qdqwdqwdqw1212</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
almost everything is done
</commit_message>
<xml_diff>
--- a/CLIENT_FEEDBACK.xlsx
+++ b/CLIENT_FEEDBACK.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -774,6 +774,336 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-02-18 08:33:54</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>123123</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>123123</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-18 08:57:09</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>123123qwdqwd</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1231232112312qwdqwdwqdqwdqwdqwdwqdqwdqwdqwdqwdqwdqwdqd</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-18 08:59:51</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>123123qwdqwdqwd</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>12312312</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:00:18</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>qwdqwdqw</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>121221</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:04:31</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>123123qwdqwdqw</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>123123qwdqwdqwdqwdqwdwqdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwdqwd</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:06:27</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>improvement</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>wqdqwdqw</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>12312312312312312312312312312312312312321321321312312312312d</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>admin@example.com</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
i think i js need to change fonts then it shld be done
</commit_message>
<xml_diff>
--- a/CLIENT_FEEDBACK.xlsx
+++ b/CLIENT_FEEDBACK.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1104,6 +1104,61 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-02-18 10:28:55</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>improvement</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>12ddqw</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1231212312312321312321312312312312312312321321312312312312dwqdd</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IM FUCKING DONE HELL YEAH
</commit_message>
<xml_diff>
--- a/CLIENT_FEEDBACK.xlsx
+++ b/CLIENT_FEEDBACK.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1159,6 +1159,61 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-02-18 12:26:50</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>urmom</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>urmommansdasndasdsadashdasdasdasdasdasdasddasasdasdasdas</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>admin@example.com</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>